<commit_message>
update excel and data
</commit_message>
<xml_diff>
--- a/Cambium_Import_Details.xlsx
+++ b/Cambium_Import_Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\czad\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73996E66-ADD3-48FC-BA31-EA937A412FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A4C236-A017-4ECE-8892-53621287C56D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{42E993CD-9B70-4509-B668-6EEF51FEBD70}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1619" uniqueCount="1213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1636" uniqueCount="1230">
   <si>
     <t>SR NO</t>
   </si>
@@ -3696,6 +3696,57 @@
   </si>
   <si>
     <t>B0GN86G345</t>
+  </si>
+  <si>
+    <t>B0GW8Z556N</t>
+  </si>
+  <si>
+    <t>B0GW8VBCBL</t>
+  </si>
+  <si>
+    <t>B0GW9461N5</t>
+  </si>
+  <si>
+    <t>B0GW8YC59C</t>
+  </si>
+  <si>
+    <t>B0GW92TVVC</t>
+  </si>
+  <si>
+    <t>B0GW8XGPB2</t>
+  </si>
+  <si>
+    <t>B0GW92TQGV</t>
+  </si>
+  <si>
+    <t>B0GW96SHSK</t>
+  </si>
+  <si>
+    <t>B0GW92TTMS</t>
+  </si>
+  <si>
+    <t>B0GW92316G</t>
+  </si>
+  <si>
+    <t>B0GW96CQMG</t>
+  </si>
+  <si>
+    <t>B0GW8R2RYM</t>
+  </si>
+  <si>
+    <t>B0GW8ZQRFK</t>
+  </si>
+  <si>
+    <t>B0GTZND3ZN</t>
+  </si>
+  <si>
+    <t>B0GTZJF142</t>
+  </si>
+  <si>
+    <t>B0GTZLGPFR</t>
+  </si>
+  <si>
+    <t>B0GTZ9X8Q2</t>
   </si>
 </sst>
 </file>
@@ -3805,7 +3856,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3827,6 +3878,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3835,6 +3889,16 @@
   <dxfs count="196">
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -3847,6 +3911,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -3919,6 +4003,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4003,6 +4107,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4027,66 +4141,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4099,6 +4153,56 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4161,16 +4265,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4215,46 +4309,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4339,6 +4393,66 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4363,96 +4477,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4495,6 +4519,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4519,6 +4573,66 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4571,26 +4685,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color rgb="FF9C0006"/>
@@ -4638,6 +4732,356 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
@@ -4659,366 +5103,6 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -5729,36 +5813,6 @@
       <font>
         <condense val="0"/>
         <extend val="0"/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -10042,10 +10096,10 @@
         <v>413</v>
       </c>
       <c r="F137" s="7">
-        <v>0</v>
+        <v>522</v>
       </c>
       <c r="G137" s="8">
-        <v>1994</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="138" spans="1:7">
@@ -10686,10 +10740,10 @@
         <v>497</v>
       </c>
       <c r="F165" s="7">
-        <v>0</v>
+        <v>1002</v>
       </c>
       <c r="G165" s="8">
-        <v>1002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166" spans="1:7">
@@ -15713,7 +15767,9 @@
       <c r="C384" s="4" t="s">
         <v>1170</v>
       </c>
-      <c r="D384" s="3"/>
+      <c r="D384" s="9" t="s">
+        <v>1213</v>
+      </c>
       <c r="E384" s="4" t="s">
         <v>1153</v>
       </c>
@@ -15734,7 +15790,9 @@
       <c r="C385" s="4" t="s">
         <v>1171</v>
       </c>
-      <c r="D385" s="3"/>
+      <c r="D385" s="9" t="s">
+        <v>1214</v>
+      </c>
       <c r="E385" s="4" t="s">
         <v>1154</v>
       </c>
@@ -15755,7 +15813,9 @@
       <c r="C386" s="4" t="s">
         <v>1172</v>
       </c>
-      <c r="D386" s="3"/>
+      <c r="D386" s="9" t="s">
+        <v>1215</v>
+      </c>
       <c r="E386" s="4" t="s">
         <v>1155</v>
       </c>
@@ -15776,7 +15836,9 @@
       <c r="C387" s="4" t="s">
         <v>1173</v>
       </c>
-      <c r="D387" s="3"/>
+      <c r="D387" s="9" t="s">
+        <v>1216</v>
+      </c>
       <c r="E387" s="4" t="s">
         <v>1156</v>
       </c>
@@ -15797,7 +15859,9 @@
       <c r="C388" s="4" t="s">
         <v>1174</v>
       </c>
-      <c r="D388" s="3"/>
+      <c r="D388" s="9" t="s">
+        <v>1217</v>
+      </c>
       <c r="E388" s="4" t="s">
         <v>1157</v>
       </c>
@@ -15818,7 +15882,9 @@
       <c r="C389" s="4" t="s">
         <v>1175</v>
       </c>
-      <c r="D389" s="3"/>
+      <c r="D389" s="9" t="s">
+        <v>1218</v>
+      </c>
       <c r="E389" s="4" t="s">
         <v>1158</v>
       </c>
@@ -15839,7 +15905,9 @@
       <c r="C390" s="4" t="s">
         <v>1176</v>
       </c>
-      <c r="D390" s="3"/>
+      <c r="D390" s="9" t="s">
+        <v>1219</v>
+      </c>
       <c r="E390" s="4" t="s">
         <v>1159</v>
       </c>
@@ -15860,7 +15928,9 @@
       <c r="C391" s="4" t="s">
         <v>1177</v>
       </c>
-      <c r="D391" s="3"/>
+      <c r="D391" s="9" t="s">
+        <v>1220</v>
+      </c>
       <c r="E391" s="4" t="s">
         <v>1160</v>
       </c>
@@ -15881,7 +15951,9 @@
       <c r="C392" s="4" t="s">
         <v>1178</v>
       </c>
-      <c r="D392" s="3"/>
+      <c r="D392" s="9" t="s">
+        <v>1221</v>
+      </c>
       <c r="E392" s="4" t="s">
         <v>1161</v>
       </c>
@@ -15902,7 +15974,9 @@
       <c r="C393" s="4" t="s">
         <v>1179</v>
       </c>
-      <c r="D393" s="3"/>
+      <c r="D393" s="9" t="s">
+        <v>1222</v>
+      </c>
       <c r="E393" s="4" t="s">
         <v>1162</v>
       </c>
@@ -15923,7 +15997,9 @@
       <c r="C394" s="4" t="s">
         <v>1180</v>
       </c>
-      <c r="D394" s="3"/>
+      <c r="D394" s="9" t="s">
+        <v>1223</v>
+      </c>
       <c r="E394" s="4" t="s">
         <v>1163</v>
       </c>
@@ -15944,7 +16020,9 @@
       <c r="C395" s="4" t="s">
         <v>1181</v>
       </c>
-      <c r="D395" s="3"/>
+      <c r="D395" s="9" t="s">
+        <v>1224</v>
+      </c>
       <c r="E395" s="4" t="s">
         <v>1164</v>
       </c>
@@ -15965,7 +16043,9 @@
       <c r="C396" s="4" t="s">
         <v>1182</v>
       </c>
-      <c r="D396" s="3"/>
+      <c r="D396" s="9" t="s">
+        <v>1225</v>
+      </c>
       <c r="E396" s="4" t="s">
         <v>1165</v>
       </c>
@@ -15986,7 +16066,9 @@
       <c r="C397" s="4" t="s">
         <v>1183</v>
       </c>
-      <c r="D397" s="3"/>
+      <c r="D397" s="9" t="s">
+        <v>1226</v>
+      </c>
       <c r="E397" s="4" t="s">
         <v>1166</v>
       </c>
@@ -16007,7 +16089,9 @@
       <c r="C398" s="4" t="s">
         <v>1184</v>
       </c>
-      <c r="D398" s="3"/>
+      <c r="D398" s="9" t="s">
+        <v>1227</v>
+      </c>
       <c r="E398" s="4" t="s">
         <v>1167</v>
       </c>
@@ -16028,7 +16112,9 @@
       <c r="C399" s="4" t="s">
         <v>1185</v>
       </c>
-      <c r="D399" s="3"/>
+      <c r="D399" s="9" t="s">
+        <v>1228</v>
+      </c>
       <c r="E399" s="4" t="s">
         <v>1168</v>
       </c>
@@ -16049,7 +16135,9 @@
       <c r="C400" s="4" t="s">
         <v>1186</v>
       </c>
-      <c r="D400" s="3"/>
+      <c r="D400" s="9" t="s">
+        <v>1229</v>
+      </c>
       <c r="E400" s="4" t="s">
         <v>1169</v>
       </c>
@@ -16101,10 +16189,10 @@
         <v>1191</v>
       </c>
       <c r="F402" s="7">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="G402" s="7">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="403" spans="1:7">
@@ -16282,6 +16370,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G410" xr:uid="{2638B9F0-C254-4E3B-92A1-1C14FA755F6E}"/>
   <conditionalFormatting sqref="C1:C152 C154:C358">
     <cfRule type="duplicateValues" dxfId="195" priority="267"/>
   </conditionalFormatting>
@@ -16293,24 +16382,24 @@
     <cfRule type="duplicateValues" dxfId="192" priority="251"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C291">
-    <cfRule type="duplicateValues" dxfId="191" priority="240"/>
-    <cfRule type="duplicateValues" dxfId="190" priority="241"/>
-    <cfRule type="duplicateValues" dxfId="189" priority="242"/>
-    <cfRule type="duplicateValues" dxfId="188" priority="243"/>
-    <cfRule type="duplicateValues" dxfId="187" priority="244"/>
-    <cfRule type="duplicateValues" dxfId="186" priority="245"/>
-    <cfRule type="duplicateValues" dxfId="185" priority="246" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="184" priority="247" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="191" priority="243"/>
+    <cfRule type="duplicateValues" dxfId="190" priority="244"/>
+    <cfRule type="duplicateValues" dxfId="189" priority="245"/>
+    <cfRule type="duplicateValues" dxfId="188" priority="246" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="187" priority="247" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="186" priority="240"/>
+    <cfRule type="duplicateValues" dxfId="185" priority="241"/>
+    <cfRule type="duplicateValues" dxfId="184" priority="242"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C330:C333">
     <cfRule type="duplicateValues" dxfId="183" priority="239"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21">
-    <cfRule type="duplicateValues" dxfId="182" priority="160"/>
-    <cfRule type="duplicateValues" dxfId="181" priority="161"/>
+    <cfRule type="duplicateValues" dxfId="182" priority="164" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="181" priority="163" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="180" priority="162" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="179" priority="163" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="178" priority="164" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="179" priority="161"/>
+    <cfRule type="duplicateValues" dxfId="178" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30">
     <cfRule type="duplicateValues" dxfId="177" priority="165"/>
@@ -16324,136 +16413,136 @@
     <cfRule type="duplicateValues" dxfId="171" priority="187" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E31:E61 E22:E29 E7:E20">
-    <cfRule type="duplicateValues" dxfId="170" priority="188"/>
-    <cfRule type="duplicateValues" dxfId="169" priority="189" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="170" priority="189" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="169" priority="188"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E37:E56">
     <cfRule type="duplicateValues" dxfId="168" priority="185" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E111">
-    <cfRule type="duplicateValues" dxfId="167" priority="150"/>
-    <cfRule type="duplicateValues" dxfId="166" priority="151"/>
+    <cfRule type="duplicateValues" dxfId="167" priority="154" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="166" priority="153" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="165" priority="152" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="164" priority="153" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="163" priority="154" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="164" priority="150"/>
+    <cfRule type="duplicateValues" dxfId="163" priority="151"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E112:E114 E89:E110 E62:E64">
-    <cfRule type="duplicateValues" dxfId="162" priority="258"/>
-    <cfRule type="duplicateValues" dxfId="161" priority="259" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="162" priority="259" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="161" priority="258"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E112:E114">
-    <cfRule type="duplicateValues" dxfId="160" priority="264"/>
-    <cfRule type="duplicateValues" dxfId="159" priority="265" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="160" priority="265" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="159" priority="264"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E115:E140">
-    <cfRule type="duplicateValues" dxfId="158" priority="132"/>
-    <cfRule type="duplicateValues" dxfId="157" priority="133"/>
-    <cfRule type="duplicateValues" dxfId="156" priority="134" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="155" priority="135" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="154" priority="136" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="158" priority="136" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="157" priority="135" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="156" priority="132"/>
+    <cfRule type="duplicateValues" dxfId="155" priority="133"/>
+    <cfRule type="duplicateValues" dxfId="154" priority="134" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E155:E165">
-    <cfRule type="duplicateValues" dxfId="153" priority="117"/>
-    <cfRule type="duplicateValues" dxfId="152" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="153" priority="121" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="152" priority="120" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="151" priority="119" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="150" priority="120" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="149" priority="121" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="150" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="149" priority="117"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E166:E170 E172:E173">
-    <cfRule type="duplicateValues" dxfId="148" priority="112"/>
-    <cfRule type="duplicateValues" dxfId="147" priority="113"/>
-    <cfRule type="duplicateValues" dxfId="146" priority="114" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="145" priority="115" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="144" priority="116" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="148" priority="115" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="147" priority="116" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="146" priority="112"/>
+    <cfRule type="duplicateValues" dxfId="145" priority="113"/>
+    <cfRule type="duplicateValues" dxfId="144" priority="114" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E171">
-    <cfRule type="duplicateValues" dxfId="143" priority="170"/>
-    <cfRule type="duplicateValues" dxfId="142" priority="171"/>
-    <cfRule type="duplicateValues" dxfId="141" priority="172" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="140" priority="173" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="139" priority="174" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="174" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="172" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="173" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E174:E181">
-    <cfRule type="duplicateValues" dxfId="138" priority="107"/>
-    <cfRule type="duplicateValues" dxfId="137" priority="108"/>
-    <cfRule type="duplicateValues" dxfId="136" priority="109" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="135" priority="110" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="134" priority="111" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="109" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="107"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="108"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="111" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="110" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E182">
-    <cfRule type="duplicateValues" dxfId="133" priority="104" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="132" priority="105" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="131" priority="106" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="106" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="104" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="105" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E183:E188">
-    <cfRule type="duplicateValues" dxfId="130" priority="155"/>
-    <cfRule type="duplicateValues" dxfId="129" priority="156"/>
-    <cfRule type="duplicateValues" dxfId="128" priority="157" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="156"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="157" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="159" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="127" priority="158" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="126" priority="159" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="155"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E206:E219">
-    <cfRule type="duplicateValues" dxfId="125" priority="99"/>
-    <cfRule type="duplicateValues" dxfId="124" priority="100"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="103" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="99"/>
     <cfRule type="duplicateValues" dxfId="123" priority="101" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="122" priority="102" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="121" priority="103" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="100"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E220:E221">
-    <cfRule type="duplicateValues" dxfId="120" priority="252"/>
-    <cfRule type="duplicateValues" dxfId="119" priority="253"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="256" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="255" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="118" priority="254" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="117" priority="255" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="116" priority="256" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="253"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="252"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E222:E227">
     <cfRule type="duplicateValues" dxfId="115" priority="257"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E235:E239">
-    <cfRule type="duplicateValues" dxfId="114" priority="89"/>
-    <cfRule type="duplicateValues" dxfId="113" priority="90"/>
-    <cfRule type="duplicateValues" dxfId="112" priority="91" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="93" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="111" priority="92" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="110" priority="93" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="91" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E243:E246">
     <cfRule type="duplicateValues" dxfId="109" priority="84"/>
     <cfRule type="duplicateValues" dxfId="108" priority="85"/>
-    <cfRule type="duplicateValues" dxfId="107" priority="86" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="106" priority="87" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="105" priority="88" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="88" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="86" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="87" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E247:E252">
-    <cfRule type="duplicateValues" dxfId="104" priority="79"/>
-    <cfRule type="duplicateValues" dxfId="103" priority="80"/>
-    <cfRule type="duplicateValues" dxfId="102" priority="81" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="101" priority="82" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="100" priority="83" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="81" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="83" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="82" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="80"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E254">
-    <cfRule type="duplicateValues" dxfId="99" priority="180"/>
-    <cfRule type="duplicateValues" dxfId="98" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="184" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="183" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="97" priority="182" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="96" priority="183" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="95" priority="184" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="180"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E255:E260">
-    <cfRule type="duplicateValues" dxfId="94" priority="69"/>
-    <cfRule type="duplicateValues" dxfId="93" priority="70"/>
-    <cfRule type="duplicateValues" dxfId="92" priority="71" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="91" priority="72" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="90" priority="73" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="73" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="71" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="72" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E261:E266">
-    <cfRule type="duplicateValues" dxfId="89" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="66" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="88" priority="65"/>
-    <cfRule type="duplicateValues" dxfId="87" priority="66" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="64"/>
     <cfRule type="duplicateValues" dxfId="86" priority="67" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="85" priority="68" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E267:E281">
-    <cfRule type="duplicateValues" dxfId="84" priority="59"/>
-    <cfRule type="duplicateValues" dxfId="83" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="59"/>
     <cfRule type="duplicateValues" dxfId="82" priority="61" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="81" priority="62" stopIfTrue="1"/>
     <cfRule type="duplicateValues" dxfId="80" priority="63" stopIfTrue="1"/>
@@ -16461,21 +16550,21 @@
   <conditionalFormatting sqref="E282:E291">
     <cfRule type="duplicateValues" dxfId="79" priority="51"/>
     <cfRule type="duplicateValues" dxfId="78" priority="52"/>
-    <cfRule type="duplicateValues" dxfId="77" priority="53"/>
-    <cfRule type="duplicateValues" dxfId="76" priority="54"/>
-    <cfRule type="duplicateValues" dxfId="75" priority="55"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="56"/>
-    <cfRule type="duplicateValues" dxfId="73" priority="57" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="72" priority="58" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="58" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="57" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E292:E295">
-    <cfRule type="duplicateValues" dxfId="71" priority="43"/>
-    <cfRule type="duplicateValues" dxfId="70" priority="44"/>
-    <cfRule type="duplicateValues" dxfId="69" priority="45"/>
-    <cfRule type="duplicateValues" dxfId="68" priority="46"/>
-    <cfRule type="duplicateValues" dxfId="67" priority="47"/>
-    <cfRule type="duplicateValues" dxfId="66" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="49" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="49" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="45"/>
     <cfRule type="duplicateValues" dxfId="64" priority="50" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E296:E297">
@@ -16485,20 +16574,20 @@
     <cfRule type="duplicateValues" dxfId="60" priority="213"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E304:E308">
-    <cfRule type="duplicateValues" dxfId="59" priority="214" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="58" priority="215"/>
-    <cfRule type="duplicateValues" dxfId="57" priority="216"/>
-    <cfRule type="duplicateValues" dxfId="56" priority="217"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="217"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="216"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="215"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="214" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E309:E314">
-    <cfRule type="duplicateValues" dxfId="55" priority="218"/>
-    <cfRule type="duplicateValues" dxfId="54" priority="219"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="220"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="221"/>
-    <cfRule type="duplicateValues" dxfId="51" priority="222"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="223"/>
-    <cfRule type="duplicateValues" dxfId="49" priority="224" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="225" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="225" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="224" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="219"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="220"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="221"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="222"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="223"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="218"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E315:E326">
     <cfRule type="duplicateValues" dxfId="47" priority="231"/>
@@ -16507,58 +16596,58 @@
     <cfRule type="duplicateValues" dxfId="44" priority="234"/>
     <cfRule type="duplicateValues" dxfId="43" priority="235"/>
     <cfRule type="duplicateValues" dxfId="42" priority="236"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="237" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="40" priority="238" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="238" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="237" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E327">
-    <cfRule type="duplicateValues" dxfId="39" priority="35"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="37" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="38"/>
-    <cfRule type="duplicateValues" dxfId="35" priority="39"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="40"/>
-    <cfRule type="duplicateValues" dxfId="33" priority="41" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="42" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="42" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="41" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E328">
-    <cfRule type="duplicateValues" dxfId="31" priority="27"/>
-    <cfRule type="duplicateValues" dxfId="30" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="28" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="31"/>
-    <cfRule type="duplicateValues" dxfId="26" priority="32"/>
-    <cfRule type="duplicateValues" dxfId="25" priority="33" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="33" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="29"/>
     <cfRule type="duplicateValues" dxfId="24" priority="34" stopIfTrue="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E329">
-    <cfRule type="duplicateValues" dxfId="23" priority="19"/>
-    <cfRule type="duplicateValues" dxfId="22" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="21"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
-    <cfRule type="duplicateValues" dxfId="19" priority="23"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="24"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="25" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="26" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="26" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="25" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E331:E357">
     <cfRule type="duplicateValues" dxfId="15" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="10" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="9" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="8"/>
     <cfRule type="duplicateValues" dxfId="11" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="9" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="10" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E359:E410">
-    <cfRule type="duplicateValues" dxfId="7" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="15"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="18" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="11"/>
     <cfRule type="duplicateValues" dxfId="1" priority="17" stopIfTrue="1"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="18" stopIfTrue="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="13"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update excel and add gitignore
</commit_message>
<xml_diff>
--- a/Cambium_Import_Details.xlsx
+++ b/Cambium_Import_Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\czad\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A4C236-A017-4ECE-8892-53621287C56D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601AE856-24C0-4AC6-8E7B-B084A9CCF1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{42E993CD-9B70-4509-B668-6EEF51FEBD70}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$410</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$412</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1636" uniqueCount="1230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1648" uniqueCount="1240">
   <si>
     <t>SR NO</t>
   </si>
@@ -3698,6 +3698,9 @@
     <t>B0GN86G345</t>
   </si>
   <si>
+    <t>Remarks</t>
+  </si>
+  <si>
     <t>B0GW8Z556N</t>
   </si>
   <si>
@@ -3747,6 +3750,33 @@
   </si>
   <si>
     <t>B0GTZ9X8Q2</t>
+  </si>
+  <si>
+    <t>FBA80109</t>
+  </si>
+  <si>
+    <t>FBA80110</t>
+  </si>
+  <si>
+    <t>M5</t>
+  </si>
+  <si>
+    <t>X5</t>
+  </si>
+  <si>
+    <t>B0GXPBHDRF</t>
+  </si>
+  <si>
+    <t>B0GXP97CZG</t>
+  </si>
+  <si>
+    <t>B0GXP7LJ75</t>
+  </si>
+  <si>
+    <t>B0GN94YDY2</t>
+  </si>
+  <si>
+    <t>B0GN8WW6BC</t>
   </si>
 </sst>
 </file>
@@ -3808,7 +3838,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3827,8 +3857,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -3851,12 +3887,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3878,7 +3925,11 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6936,7 +6987,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2638B9F0-C254-4E3B-92A1-1C14FA755F6E}">
-  <dimension ref="A1:G410"/>
+  <dimension ref="A1:H412"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -6948,7 +6999,7 @@
     <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -6970,8 +7021,11 @@
       <c r="G1" s="5" t="s">
         <v>1139</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="9" t="s">
+        <v>1213</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -6994,7 +7048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:8">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -7017,7 +7071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:8">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -7040,7 +7094,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:8">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -7063,7 +7117,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:8">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -7086,7 +7140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:8">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -7109,7 +7163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:8">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -7132,7 +7186,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:8">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -7155,7 +7209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:8">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -7178,7 +7232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:8">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -7201,7 +7255,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:8">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -7224,7 +7278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:8">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -7247,7 +7301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:8">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -7270,7 +7324,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:8">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -7293,7 +7347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:8">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -9547,7 +9601,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="7">
-        <v>0</v>
+        <v>504</v>
       </c>
     </row>
     <row r="114" spans="1:7">
@@ -9895,7 +9949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:7">
+    <row r="129" spans="1:8">
       <c r="A129" s="1">
         <v>128</v>
       </c>
@@ -9918,7 +9972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:7">
+    <row r="130" spans="1:8">
       <c r="A130" s="1">
         <v>129</v>
       </c>
@@ -9941,7 +9995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="16.8">
+    <row r="131" spans="1:8" ht="16.8">
       <c r="A131" s="1">
         <v>130</v>
       </c>
@@ -9964,7 +10018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:7">
+    <row r="132" spans="1:8">
       <c r="A132" s="1">
         <v>131</v>
       </c>
@@ -9987,7 +10041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:7">
+    <row r="133" spans="1:8">
       <c r="A133" s="1">
         <v>132</v>
       </c>
@@ -10010,7 +10064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:7">
+    <row r="134" spans="1:8">
       <c r="A134" s="1">
         <v>133</v>
       </c>
@@ -10033,7 +10087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:7">
+    <row r="135" spans="1:8">
       <c r="A135" s="1">
         <v>134</v>
       </c>
@@ -10056,7 +10110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:7">
+    <row r="136" spans="1:8">
       <c r="A136" s="1">
         <v>135</v>
       </c>
@@ -10079,7 +10133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:7">
+    <row r="137" spans="1:8">
       <c r="A137" s="1">
         <v>136</v>
       </c>
@@ -10101,8 +10155,9 @@
       <c r="G137" s="8">
         <v>1472</v>
       </c>
-    </row>
-    <row r="138" spans="1:7">
+      <c r="H137" s="10"/>
+    </row>
+    <row r="138" spans="1:8">
       <c r="A138" s="1">
         <v>137</v>
       </c>
@@ -10125,7 +10180,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="139" spans="1:7">
+    <row r="139" spans="1:8">
       <c r="A139" s="1">
         <v>138</v>
       </c>
@@ -10148,7 +10203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:7">
+    <row r="140" spans="1:8">
       <c r="A140" s="1">
         <v>139</v>
       </c>
@@ -10171,7 +10226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:7">
+    <row r="141" spans="1:8">
       <c r="A141" s="1">
         <v>140</v>
       </c>
@@ -10194,7 +10249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:7">
+    <row r="142" spans="1:8">
       <c r="A142" s="1">
         <v>141</v>
       </c>
@@ -10217,7 +10272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:7">
+    <row r="143" spans="1:8">
       <c r="A143" s="1">
         <v>142</v>
       </c>
@@ -10240,7 +10295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:7">
+    <row r="144" spans="1:8">
       <c r="A144" s="1">
         <v>143</v>
       </c>
@@ -10421,7 +10476,7 @@
         <v>0</v>
       </c>
       <c r="G151" s="7">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="152" spans="1:7">
@@ -11249,7 +11304,7 @@
         <v>0</v>
       </c>
       <c r="G187" s="7">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="188" spans="1:7">
@@ -15767,8 +15822,8 @@
       <c r="C384" s="4" t="s">
         <v>1170</v>
       </c>
-      <c r="D384" s="9" t="s">
-        <v>1213</v>
+      <c r="D384" s="11" t="s">
+        <v>1214</v>
       </c>
       <c r="E384" s="4" t="s">
         <v>1153</v>
@@ -15790,8 +15845,8 @@
       <c r="C385" s="4" t="s">
         <v>1171</v>
       </c>
-      <c r="D385" s="9" t="s">
-        <v>1214</v>
+      <c r="D385" s="11" t="s">
+        <v>1215</v>
       </c>
       <c r="E385" s="4" t="s">
         <v>1154</v>
@@ -15813,8 +15868,8 @@
       <c r="C386" s="4" t="s">
         <v>1172</v>
       </c>
-      <c r="D386" s="9" t="s">
-        <v>1215</v>
+      <c r="D386" s="11" t="s">
+        <v>1216</v>
       </c>
       <c r="E386" s="4" t="s">
         <v>1155</v>
@@ -15836,8 +15891,8 @@
       <c r="C387" s="4" t="s">
         <v>1173</v>
       </c>
-      <c r="D387" s="9" t="s">
-        <v>1216</v>
+      <c r="D387" s="11" t="s">
+        <v>1217</v>
       </c>
       <c r="E387" s="4" t="s">
         <v>1156</v>
@@ -15859,8 +15914,8 @@
       <c r="C388" s="4" t="s">
         <v>1174</v>
       </c>
-      <c r="D388" s="9" t="s">
-        <v>1217</v>
+      <c r="D388" s="11" t="s">
+        <v>1218</v>
       </c>
       <c r="E388" s="4" t="s">
         <v>1157</v>
@@ -15882,8 +15937,8 @@
       <c r="C389" s="4" t="s">
         <v>1175</v>
       </c>
-      <c r="D389" s="9" t="s">
-        <v>1218</v>
+      <c r="D389" s="11" t="s">
+        <v>1219</v>
       </c>
       <c r="E389" s="4" t="s">
         <v>1158</v>
@@ -15905,8 +15960,8 @@
       <c r="C390" s="4" t="s">
         <v>1176</v>
       </c>
-      <c r="D390" s="9" t="s">
-        <v>1219</v>
+      <c r="D390" s="11" t="s">
+        <v>1220</v>
       </c>
       <c r="E390" s="4" t="s">
         <v>1159</v>
@@ -15928,8 +15983,8 @@
       <c r="C391" s="4" t="s">
         <v>1177</v>
       </c>
-      <c r="D391" s="9" t="s">
-        <v>1220</v>
+      <c r="D391" s="11" t="s">
+        <v>1221</v>
       </c>
       <c r="E391" s="4" t="s">
         <v>1160</v>
@@ -15951,8 +16006,8 @@
       <c r="C392" s="4" t="s">
         <v>1178</v>
       </c>
-      <c r="D392" s="9" t="s">
-        <v>1221</v>
+      <c r="D392" s="11" t="s">
+        <v>1222</v>
       </c>
       <c r="E392" s="4" t="s">
         <v>1161</v>
@@ -15974,8 +16029,8 @@
       <c r="C393" s="4" t="s">
         <v>1179</v>
       </c>
-      <c r="D393" s="9" t="s">
-        <v>1222</v>
+      <c r="D393" s="11" t="s">
+        <v>1223</v>
       </c>
       <c r="E393" s="4" t="s">
         <v>1162</v>
@@ -15997,8 +16052,8 @@
       <c r="C394" s="4" t="s">
         <v>1180</v>
       </c>
-      <c r="D394" s="9" t="s">
-        <v>1223</v>
+      <c r="D394" s="11" t="s">
+        <v>1224</v>
       </c>
       <c r="E394" s="4" t="s">
         <v>1163</v>
@@ -16020,8 +16075,8 @@
       <c r="C395" s="4" t="s">
         <v>1181</v>
       </c>
-      <c r="D395" s="9" t="s">
-        <v>1224</v>
+      <c r="D395" s="11" t="s">
+        <v>1225</v>
       </c>
       <c r="E395" s="4" t="s">
         <v>1164</v>
@@ -16043,8 +16098,8 @@
       <c r="C396" s="4" t="s">
         <v>1182</v>
       </c>
-      <c r="D396" s="9" t="s">
-        <v>1225</v>
+      <c r="D396" s="11" t="s">
+        <v>1226</v>
       </c>
       <c r="E396" s="4" t="s">
         <v>1165</v>
@@ -16066,8 +16121,8 @@
       <c r="C397" s="4" t="s">
         <v>1183</v>
       </c>
-      <c r="D397" s="9" t="s">
-        <v>1226</v>
+      <c r="D397" s="11" t="s">
+        <v>1227</v>
       </c>
       <c r="E397" s="4" t="s">
         <v>1166</v>
@@ -16089,8 +16144,8 @@
       <c r="C398" s="4" t="s">
         <v>1184</v>
       </c>
-      <c r="D398" s="9" t="s">
-        <v>1227</v>
+      <c r="D398" s="11" t="s">
+        <v>1228</v>
       </c>
       <c r="E398" s="4" t="s">
         <v>1167</v>
@@ -16112,8 +16167,8 @@
       <c r="C399" s="4" t="s">
         <v>1185</v>
       </c>
-      <c r="D399" s="9" t="s">
-        <v>1228</v>
+      <c r="D399" s="11" t="s">
+        <v>1229</v>
       </c>
       <c r="E399" s="4" t="s">
         <v>1168</v>
@@ -16135,8 +16190,8 @@
       <c r="C400" s="4" t="s">
         <v>1186</v>
       </c>
-      <c r="D400" s="9" t="s">
-        <v>1229</v>
+      <c r="D400" s="11" t="s">
+        <v>1230</v>
       </c>
       <c r="E400" s="4" t="s">
         <v>1169</v>
@@ -16274,7 +16329,9 @@
       <c r="C406" s="4" t="s">
         <v>1205</v>
       </c>
-      <c r="D406" s="3"/>
+      <c r="D406" s="3" t="s">
+        <v>1238</v>
+      </c>
       <c r="E406" s="4" t="s">
         <v>1195</v>
       </c>
@@ -16295,7 +16352,9 @@
       <c r="C407" s="4" t="s">
         <v>1206</v>
       </c>
-      <c r="D407" s="3"/>
+      <c r="D407" s="3" t="s">
+        <v>1239</v>
+      </c>
       <c r="E407" s="4" t="s">
         <v>1196</v>
       </c>
@@ -16316,7 +16375,9 @@
       <c r="C408" s="4" t="s">
         <v>1199</v>
       </c>
-      <c r="D408" s="3"/>
+      <c r="D408" s="3" t="s">
+        <v>1235</v>
+      </c>
       <c r="E408" s="4" t="s">
         <v>1197</v>
       </c>
@@ -16337,7 +16398,9 @@
       <c r="C409" s="4" t="s">
         <v>1200</v>
       </c>
-      <c r="D409" s="3"/>
+      <c r="D409" s="3" t="s">
+        <v>1236</v>
+      </c>
       <c r="E409" s="4" t="s">
         <v>1198</v>
       </c>
@@ -16358,7 +16421,9 @@
       <c r="C410" s="4" t="s">
         <v>1208</v>
       </c>
-      <c r="D410" s="3"/>
+      <c r="D410" s="3" t="s">
+        <v>1237</v>
+      </c>
       <c r="E410" s="4" t="s">
         <v>1207</v>
       </c>
@@ -16369,8 +16434,49 @@
         <v>0</v>
       </c>
     </row>
+    <row r="411" spans="1:7">
+      <c r="A411" s="1">
+        <v>410</v>
+      </c>
+      <c r="B411" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C411" s="4" t="s">
+        <v>1231</v>
+      </c>
+      <c r="D411" s="3"/>
+      <c r="E411" s="4" t="s">
+        <v>1233</v>
+      </c>
+      <c r="F411" s="7">
+        <v>0</v>
+      </c>
+      <c r="G411" s="7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="412" spans="1:7">
+      <c r="A412" s="1">
+        <v>411</v>
+      </c>
+      <c r="B412" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C412" s="4" t="s">
+        <v>1232</v>
+      </c>
+      <c r="D412" s="3"/>
+      <c r="E412" s="4" t="s">
+        <v>1234</v>
+      </c>
+      <c r="F412" s="7">
+        <v>0</v>
+      </c>
+      <c r="G412" s="7">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G410" xr:uid="{2638B9F0-C254-4E3B-92A1-1C14FA755F6E}"/>
   <conditionalFormatting sqref="C1:C152 C154:C358">
     <cfRule type="duplicateValues" dxfId="195" priority="267"/>
   </conditionalFormatting>
@@ -16639,7 +16745,7 @@
     <cfRule type="duplicateValues" dxfId="9" priority="5"/>
     <cfRule type="duplicateValues" dxfId="8" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E359:E410">
+  <conditionalFormatting sqref="E359:E412">
     <cfRule type="duplicateValues" dxfId="7" priority="16"/>
     <cfRule type="duplicateValues" dxfId="6" priority="15"/>
     <cfRule type="duplicateValues" dxfId="5" priority="14"/>

</xml_diff>